<commit_message>
De-duplicate INSA courses across USM convalidation recommendations
</commit_message>
<xml_diff>
--- a/Results/convalidation_proposals.xlsx
+++ b/Results/convalidation_proposals.xlsx
@@ -9137,11 +9137,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-5-S1-EC-PRI - Industrial project</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.1559</v>
+        <v>0.0862</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>3</v>
@@ -9160,11 +9160,11 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PCO - Collective project S1</t>
+          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.1429</v>
+        <v>0.0862</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>3</v>
@@ -9183,11 +9183,11 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-PCO - Collective project S1/2</t>
+          <t>GI-3-S2-EC-GPC - Management of a machine design project</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.1307</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>4</v>
@@ -9206,14 +9206,14 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
+          <t>GI-4-S2-EC-PSM - SCADA-MES project</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.1262</v>
+        <v>0.0834</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -9229,11 +9229,11 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PRI - Industrial project</t>
+          <t>GI-4-S1-EC-PCS - Piloting and management of an industrial system</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.0862</v>
+        <v>0.079</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>3</v>
@@ -9252,14 +9252,14 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
+          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.0862</v>
+        <v>0.0759</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -9275,14 +9275,14 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-GPC - Management of a machine design project</t>
+          <t>GI-5-S1-EC-KNM - Knowledge management</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -9298,14 +9298,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-ERP - ERP Project</t>
+          <t>GI-0-S1-EC-LABECH15 - Research project for exchange student</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.0847</v>
+        <v>0.0688</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -9321,14 +9321,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.1291</v>
+        <v>0.0926</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -9344,11 +9344,11 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PCO - Collective project S1</t>
+          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.1253</v>
+        <v>0.068</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>3</v>
@@ -9367,11 +9367,11 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-PCO - Collective project S1/2</t>
+          <t>GI-3-S2-EC-GPC - Management of a machine design project</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.1121</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>4</v>
@@ -9390,14 +9390,14 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
+          <t>GI-4-S1-EC-PCS - Piloting and management of an industrial system</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.0926</v>
+        <v>0.0633</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -9413,14 +9413,14 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PRI - Industrial project</t>
+          <t>GI-3-S2-EC-RIP - Computational problem solving</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.077</v>
+        <v>0.0589</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -9436,11 +9436,11 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
+          <t>GI-3-S2-EC-GFL - Flow management</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.0757</v>
+        <v>0.0577</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>2</v>
@@ -9459,14 +9459,14 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
+          <t>GI-0-S1-EC-LABECH15 - Research project for exchange student</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.068</v>
+        <v>0.0543</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -9482,14 +9482,14 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-GPC - Management of a machine design project</t>
+          <t>GI-0-S2-EC-LABECH30 - Research project for exchange student</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0543</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -9528,11 +9528,11 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PCO - Collective project S1</t>
+          <t>GI-5-S1-EC-MGI-HU - Management for engineering</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.2313</v>
+        <v>0.2225</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>3</v>
@@ -9551,11 +9551,11 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-MGI-HU - Management for engineering</t>
+          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.2225</v>
+        <v>0.1628</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>3</v>
@@ -9574,14 +9574,14 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S1-EC-GIN - Industrial management</t>
+          <t>GI-5-S1-EC-KNM - Knowledge management</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.1815</v>
+        <v>0.1285</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -9597,14 +9597,14 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
+          <t>GI-4-S1-EC-INR - Initiation to scientific research</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.1628</v>
+        <v>0.1265</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -9620,11 +9620,11 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.1421</v>
+        <v>0.1148</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>3</v>
@@ -9643,11 +9643,11 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-KNM - Knowledge management</t>
+          <t>GI-4-S2-EC-BCG - Budget and control management</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.1285</v>
+        <v>0.0978</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>2</v>
@@ -9666,14 +9666,14 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-INR - Initiation to scientific research</t>
+          <t>GI-4-S1-EC-PCS - Piloting and management of an industrial system</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.1265</v>
+        <v>0.0906</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
@@ -9735,11 +9735,11 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-ERP - ERP Project</t>
+          <t>GI-4-S2-EC-PSM - SCADA-MES project</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.2018</v>
+        <v>0.1581</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>3</v>
@@ -9758,14 +9758,14 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S1-EC-GIN - Industrial management</t>
+          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.1726</v>
+        <v>0.1548</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -9781,14 +9781,14 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCS - Piloting and management of an industrial system</t>
+          <t>GI-3-S2-EC-CDA - Design, sizing and performance analysis of a control system</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.1671</v>
+        <v>0.1465</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -9804,11 +9804,11 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-CBD - Database design and information systems architecture</t>
+          <t>GI-5-S1-EC-IFD - Internal Supply chain and facility</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.1661</v>
+        <v>0.1336</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>3</v>
@@ -9827,14 +9827,14 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PSM - SCADA-MES project</t>
+          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.1581</v>
+        <v>0.1228</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -9850,14 +9850,14 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
+          <t>GI-3-S2-EC-GFL - Flow management</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.1548</v>
+        <v>0.1207</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -10057,11 +10057,11 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-ADM - Multicriteria decision support</t>
+          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>0.1787</v>
+        <v>0.0742</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>2</v>
@@ -10080,14 +10080,14 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
+          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>0.0742</v>
+        <v>0.0638</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
@@ -10103,14 +10103,14 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-PCO - Collective project S1</t>
+          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>0.0687</v>
+        <v>0.0521</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
@@ -10126,11 +10126,11 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
+          <t>GI-5-S1-EC-RGI - Research in Industrial Engineering</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0.0638</v>
+        <v>0.0466</v>
       </c>
       <c r="D53" s="2" t="n">
         <v>3</v>
@@ -10149,14 +10149,14 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-PCO - Collective project S1/2</t>
+          <t>GI-4-S1-EC-ORD - Scheduling</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>0.0615</v>
+        <v>0.0453</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
@@ -10172,14 +10172,14 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-4-S1-EC-ISD - Introduction to data science</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0.0562</v>
+        <v>0.0421</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
@@ -10195,14 +10195,14 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
+          <t>GI-5-S1-EC-PRI - Industrial project</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>0.0521</v>
+        <v>0.0413</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
@@ -10218,11 +10218,11 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-CBD - Database design and information systems architecture</t>
+          <t>GI-4-S1-EC-PCS - Piloting and management of an industrial system</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>0.0485</v>
+        <v>0.0401</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>3</v>
@@ -10425,14 +10425,14 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-SIE - Business Information Systems</t>
+          <t>GI-4-S2-EC-SIE - Business Information Systems</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v>0.2557</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
@@ -10448,14 +10448,14 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-SIE - Business Information Systems</t>
+          <t>GI-4-S2-EC-PSM - SCADA-MES project</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>0.2557</v>
+        <v>0.1581</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
@@ -10471,11 +10471,11 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-ERP - ERP Project</t>
+          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>0.2018</v>
+        <v>0.1548</v>
       </c>
       <c r="D68" s="2" t="n">
         <v>3</v>
@@ -10494,14 +10494,14 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S1-EC-GIN - Industrial management</t>
+          <t>GI-3-S2-EC-CDA - Design, sizing and performance analysis of a control system</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>0.1726</v>
+        <v>0.1465</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
@@ -10517,14 +10517,14 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCS - Piloting and management of an industrial system</t>
+          <t>GI-5-S1-EC-IFD - Internal Supply chain and facility</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>0.1671</v>
+        <v>0.1336</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
@@ -10540,14 +10540,14 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-CBD - Database design and information systems architecture</t>
+          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>0.1661</v>
+        <v>0.1228</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
@@ -10563,14 +10563,14 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PSM - SCADA-MES project</t>
+          <t>GI-3-S2-EC-GFL - Flow management</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>0.1581</v>
+        <v>0.1207</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
@@ -10586,14 +10586,14 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-ISC - Introduction to Supply Chain</t>
+          <t>GI-3-S2-EC-CSD - Control of dynamic systems</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>0.1548</v>
+        <v>0.1119</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
@@ -10908,14 +10908,14 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S1-EC-GIN - Industrial management</t>
+          <t>GI-3-S2-EC-RIP - Computational problem solving</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
-        <v>0.1477</v>
+        <v>0.128</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
@@ -10931,14 +10931,14 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-RIP - Computational problem solving</t>
+          <t>GI-3-S2-EC-CDA - Design, sizing and performance analysis of a control system</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
-        <v>0.128</v>
+        <v>0.1275</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
@@ -10954,11 +10954,11 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>GI-3-S2-EC-CDA - Design, sizing and performance analysis of a control system</t>
+          <t>GI-5-S1-EC-IFD - Internal Supply chain and facility</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>0.1275</v>
+        <v>0.1273</v>
       </c>
       <c r="D89" s="2" t="n">
         <v>3</v>
@@ -11060,14 +11060,14 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-5-S1-EC-PRI - Industrial project</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>15.6</v>
+        <v>8.6</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: information, plan, project.</t>
+          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: engineering, information, plan, planning, project.</t>
         </is>
       </c>
     </row>
@@ -11088,14 +11088,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S2-EC-PCO - Collective project S2/2</t>
+          <t>GI-5-S1-EC-ETH-HU - Engineering Ethics</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>12.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: plan, project.</t>
+          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: engineering, project.</t>
         </is>
       </c>
     </row>
@@ -11145,15 +11145,14 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-SIE - Business Information Systems
-GI-4-S2-EC-ERP - ERP Project</t>
+          <t>GI-4-S1-EC-SIE - Business Information Systems</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>31</v>
+        <v>25.6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -11162,7 +11161,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: business, data, decision, information, management, mining, model, planning, process, programming_code, system.</t>
+          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: business, data, information, management, mining, model, process, programming_code, system.</t>
         </is>
       </c>
     </row>
@@ -11202,14 +11201,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>GI-5-S1-EC-ADM - Multicriteria decision support</t>
+          <t>GI-4-S1-EC-BIN - Business Intelligence</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>17.9</v>
+        <v>7.4</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -11218,7 +11217,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: decision, economica.</t>
+          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: database, decision, engineering, project.</t>
         </is>
       </c>
     </row>
@@ -11259,15 +11258,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>GI-4-S1-EC-SIE - Business Information Systems
-GI-4-S2-EC-ERP - ERP Project</t>
+          <t>GI-4-S2-EC-SIE - Business Information Systems</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>31</v>
+        <v>25.6</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -11276,7 +11274,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: business, data, decision, information, management, mining, model, planning, process, programming_code, system.</t>
+          <t>Heuristic bag-of-words equivalence over extracted syllabus text. Shared topic terms: business, data, information, management, mining, model, process, programming_code, system.</t>
         </is>
       </c>
     </row>
@@ -11455,11 +11453,12 @@
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>GI-4-S1-EC-PCO (4.0 ECTS)
-GI-4-S1-EC-SIE (3.0 ECTS)</t>
+GI-4-S1-EC-SIE (3.0 ECTS)
+GI-4-S1-EC-BIN (2.0 ECTS)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -11468,7 +11467,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>36-Gestio_n-de-la-Innovacio_n, ICN-322</t>
+          <t>36-Gestio_n-de-la-Innovacio_n, ICN-322, ILN-230</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -11482,13 +11481,14 @@
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>GI-4-S2-EC-PCO (3.0 ECTS)
+GI-4-S2-EC-ISD (1.0 ECTS)
+GI-4-S2-EC-SIE (1.0 ECTS)
 GI-4-S2-EC-ERP (3.0 ECTS)
-GI-4-S2-EC-ISD (1.0 ECTS)
 GI-4-S2-EC-PCS (1.0 ECTS)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -11497,7 +11497,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>ELO-302, ELO-307, ELO-308, ICN-322, programa_download-5, ICN-345</t>
+          <t>ELO-302, programa_download-5, ICN-322, ICN-345</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -11511,13 +11511,15 @@
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>GI-5-S1-EC-PCO (3.0 ECTS)
+GI-5-S1-EC-PRI (3.0 ECTS)
+GI-5-S1-EC-ETH-HU (2.0 ECTS)
 GI-5-S1-EC-MGI-HU (3.0 ECTS)
 GI-5-S1-EC-SSC (3.0 ECTS)
 GI-5-S1-EC-ADM (2.0 ECTS)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -11526,7 +11528,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ELO-302, 36-Gestio_n-de-la-Innovacio_n, ICN-370, ILN-230, ILN-250</t>
+          <t>ELO-302, ELO-307, ELO-308, 36-Gestio_n-de-la-Innovacio_n, ICN-370, ILN-250</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>

</xml_diff>